<commit_message>
docs: regenerate KEYMAP.html and KEYMAP.xlsx from keymap
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -1910,7 +1910,7 @@
       <c r="L25" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
@@ -1956,11 +1956,7 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="L26" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L26" s="9" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1999,11 +1995,7 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="L27" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
+      <c r="L27" s="9" t="inlineStr"/>
       <c r="M27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
@@ -2760,7 +2752,7 @@
       <c r="L42" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
@@ -2802,11 +2794,7 @@
       </c>
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="9" t="inlineStr"/>
-      <c r="L43" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L43" s="9" t="inlineStr"/>
       <c r="M43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
@@ -2841,11 +2829,7 @@
       </c>
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="9" t="inlineStr"/>
-      <c r="L44" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
+      <c r="L44" s="9" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
@@ -3255,7 +3239,7 @@
       <c r="L53" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr">
@@ -3289,11 +3273,7 @@
       <c r="I54" s="9" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
       <c r="K54" s="9" t="inlineStr"/>
-      <c r="L54" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L54" s="9" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr"/>
     </row>
     <row r="55">
@@ -5289,7 +5269,7 @@
       <c r="D97" s="7" t="inlineStr">
         <is>
           <t>pos 12
-&amp;none</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
@@ -5345,7 +5325,11 @@
       </c>
       <c r="B98" s="9" t="inlineStr"/>
       <c r="C98" s="9" t="inlineStr"/>
-      <c r="D98" s="9" t="inlineStr"/>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
       <c r="E98" s="9" t="inlineStr"/>
       <c r="F98" s="9" t="inlineStr"/>
       <c r="G98" s="9" t="inlineStr"/>
@@ -5668,7 +5652,7 @@
       <c r="C106" s="7" t="inlineStr">
         <is>
           <t>pos 11
-&amp;none</t>
+&amp;mkp MB2</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -5680,7 +5664,7 @@
       <c r="E106" s="7" t="inlineStr">
         <is>
           <t>pos 13
-&amp;none</t>
+&amp;mkp MB1</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -5729,9 +5713,17 @@
         </is>
       </c>
       <c r="B107" s="9" t="inlineStr"/>
-      <c r="C107" s="9" t="inlineStr"/>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>🖱右</t>
+        </is>
+      </c>
       <c r="D107" s="9" t="inlineStr"/>
-      <c r="E107" s="9" t="inlineStr"/>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>🖱左</t>
+        </is>
+      </c>
       <c r="F107" s="9" t="inlineStr"/>
       <c r="G107" s="9" t="inlineStr"/>
       <c r="H107" s="9" t="inlineStr"/>
@@ -5764,7 +5756,7 @@
       <c r="C108" s="7" t="inlineStr">
         <is>
           <t>pos 21
-&amp;none</t>
+&amp;mkp MB5</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -5776,7 +5768,7 @@
       <c r="E108" s="7" t="inlineStr">
         <is>
           <t>pos 23
-&amp;none</t>
+&amp;mkp MB4</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -5830,9 +5822,17 @@
         </is>
       </c>
       <c r="B109" s="9" t="inlineStr"/>
-      <c r="C109" s="9" t="inlineStr"/>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>🖱進</t>
+        </is>
+      </c>
       <c r="D109" s="9" t="inlineStr"/>
-      <c r="E109" s="9" t="inlineStr"/>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>🖱戻</t>
+        </is>
+      </c>
       <c r="F109" s="9" t="inlineStr"/>
       <c r="G109" s="9" t="inlineStr"/>
       <c r="H109" s="9" t="inlineStr"/>
@@ -7338,7 +7338,7 @@
       <c r="L25" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
@@ -7384,11 +7384,7 @@
           <t>&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
-      <c r="L26" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L26" s="9" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
@@ -7427,11 +7423,7 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="L27" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
+      <c r="L27" s="9" t="inlineStr"/>
       <c r="M27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
@@ -8223,7 +8215,7 @@
       <c r="L42" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
@@ -8265,11 +8257,7 @@
       </c>
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="9" t="inlineStr"/>
-      <c r="L43" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L43" s="9" t="inlineStr"/>
       <c r="M43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
@@ -8304,11 +8292,7 @@
       </c>
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="9" t="inlineStr"/>
-      <c r="L44" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
+      <c r="L44" s="9" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
@@ -8730,7 +8714,7 @@
       <c r="L53" s="7" t="inlineStr">
         <is>
           <t>pos 40
-&amp;trans</t>
+&amp;none</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr">
@@ -8764,11 +8748,7 @@
       <c r="I54" s="9" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
       <c r="K54" s="9" t="inlineStr"/>
-      <c r="L54" s="9" t="inlineStr">
-        <is>
-          <t>▽</t>
-        </is>
-      </c>
+      <c r="L54" s="9" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr"/>
     </row>
     <row r="55">
@@ -10769,7 +10749,7 @@
       <c r="D97" s="7" t="inlineStr">
         <is>
           <t>pos 12
-&amp;none</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
@@ -10825,7 +10805,11 @@
       </c>
       <c r="B98" s="9" t="inlineStr"/>
       <c r="C98" s="9" t="inlineStr"/>
-      <c r="D98" s="9" t="inlineStr"/>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>&amp;mo MOUSE_SCROLL</t>
+        </is>
+      </c>
       <c r="E98" s="9" t="inlineStr"/>
       <c r="F98" s="9" t="inlineStr"/>
       <c r="G98" s="9" t="inlineStr"/>
@@ -11148,7 +11132,7 @@
       <c r="C106" s="7" t="inlineStr">
         <is>
           <t>pos 11
-&amp;none</t>
+&amp;mkp MB2</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -11160,7 +11144,7 @@
       <c r="E106" s="7" t="inlineStr">
         <is>
           <t>pos 13
-&amp;none</t>
+&amp;mkp MB1</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -11209,9 +11193,17 @@
         </is>
       </c>
       <c r="B107" s="9" t="inlineStr"/>
-      <c r="C107" s="9" t="inlineStr"/>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>&amp;mkp MB2</t>
+        </is>
+      </c>
       <c r="D107" s="9" t="inlineStr"/>
-      <c r="E107" s="9" t="inlineStr"/>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>&amp;mkp MB1</t>
+        </is>
+      </c>
       <c r="F107" s="9" t="inlineStr"/>
       <c r="G107" s="9" t="inlineStr"/>
       <c r="H107" s="9" t="inlineStr"/>
@@ -11244,7 +11236,7 @@
       <c r="C108" s="7" t="inlineStr">
         <is>
           <t>pos 21
-&amp;none</t>
+&amp;mkp MB5</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -11256,7 +11248,7 @@
       <c r="E108" s="7" t="inlineStr">
         <is>
           <t>pos 23
-&amp;none</t>
+&amp;mkp MB4</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -11310,9 +11302,17 @@
         </is>
       </c>
       <c r="B109" s="9" t="inlineStr"/>
-      <c r="C109" s="9" t="inlineStr"/>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>&amp;mkp MB5</t>
+        </is>
+      </c>
       <c r="D109" s="9" t="inlineStr"/>
-      <c r="E109" s="9" t="inlineStr"/>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>&amp;mkp MB4</t>
+        </is>
+      </c>
       <c r="F109" s="9" t="inlineStr"/>
       <c r="G109" s="9" t="inlineStr"/>
       <c r="H109" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
AML (マウスレイヤー) を Ctrl / Shift / Win / Alt で解除する (#38)
ryo-aoki-pc/zmk-config-LisM#22 と同じ内容 (LisM 基準)。

- excluded-positions を D / K (&mo SCRL、12 / 17) だけにする。修飾キーの位置
  (A / - / Z / / / Win / Alt) を押すと AML が切れる
- MOUSE_MOVE の修飾キーの位置を &trans にする (BASE と同じ &mt / &kp。タップで文字、
  長押しで修飾キー)
- MOUSE_SCROLL の修飾キーはそのまま。修飾キーとクリック・ホイールを組み合わせるときは
  D / K を押してから修飾キーを押す (例: D → Z → F で Shift + クリック)
- KEYMAP.html / KEYMAP.xlsx を作り直す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFG6t92cGtjhGTDoN62Yvg
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -5257,7 +5257,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -5313,7 +5313,7 @@
       <c r="M97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>LCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -5348,7 +5348,7 @@
       <c r="L98" s="9" t="inlineStr"/>
       <c r="M98" s="9" t="inlineStr">
         <is>
-          <t>RCtrl</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -5422,7 +5422,7 @@
       <c r="M99" s="7" t="inlineStr">
         <is>
           <t>pos 30
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>LShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -5449,7 +5449,7 @@
       <c r="L100" s="9" t="inlineStr"/>
       <c r="M100" s="9" t="inlineStr">
         <is>
-          <t>RShift</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5468,13 +5468,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -5536,12 +5536,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>LWin</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>LAlt</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>
@@ -10785,7 +10785,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -10841,7 +10841,7 @@
       <c r="M97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -10853,7 +10853,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -10876,7 +10876,7 @@
       <c r="L98" s="9" t="inlineStr"/>
       <c r="M98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RCTRL</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -10889,7 +10889,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -10950,7 +10950,7 @@
       <c r="M99" s="7" t="inlineStr">
         <is>
           <t>pos 30
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -10977,7 +10977,7 @@
       <c r="L100" s="9" t="inlineStr"/>
       <c r="M100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RIGHT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -10996,13 +10996,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -11064,12 +11064,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_WIN</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_ALT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>

</xml_diff>